<commit_message>
First solution for optimal matrix
</commit_message>
<xml_diff>
--- a/config/default/default2D.xlsx
+++ b/config/default/default2D.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schir\OneDrive\Studium\34_Github\TherMOS\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/TherMOS/config/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B40676-7B6B-4D44-AA0E-A3BFA33FB4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="6_{21B2E60F-E45E-4B1E-BA14-FAE5B07AE4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9A1ADF1-5FC0-4EC1-8F98-84FA382CB0E7}"/>
   <bookViews>
     <workbookView xWindow="-18120" yWindow="-2550" windowWidth="18240" windowHeight="28440" activeTab="3" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
   </bookViews>

</xml_diff>